<commit_message>
initial SIP simulation logic
</commit_message>
<xml_diff>
--- a/data/holidays_list.xlsx
+++ b/data/holidays_list.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Shrinithi Sai\Desktop\apache\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Shrinithi Sai\Desktop\sip_analysis\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{70D9D90A-7BF2-4D31-89C6-45DCD16506D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C914FED9-C713-46C3-B45B-D07477D64640}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{F7BBCC6A-4053-4BCF-9C5F-91F166136CDB}"/>
+    <workbookView xWindow="3048" yWindow="4428" windowWidth="10284" windowHeight="8532" xr2:uid="{F7BBCC6A-4053-4BCF-9C5F-91F166136CDB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -931,10 +931,10 @@
     <t>Navratri</t>
   </si>
   <si>
-    <t>DATE</t>
-  </si>
-  <si>
-    <t>HOLIDAY</t>
+    <t>Date</t>
+  </si>
+  <si>
+    <t>Holiday</t>
   </si>
 </sst>
 </file>

</xml_diff>